<commit_message>
New LRIS plan + GUI
</commit_message>
<xml_diff>
--- a/Night_plans/Keck-2026B-01/Keck_LRIS_2026Oct06_Night_plan.xlsx
+++ b/Night_plans/Keck-2026B-01/Keck_LRIS_2026Oct06_Night_plan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Observing Checklist" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="October 6th" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observing Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="October 6th" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P24"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -915,12 +915,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 min</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>19:32</t>
+          <t>19:34</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -946,27 +946,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>20.2h</t>
+          <t>20.3h</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>19:32</t>
+          <t>19:34</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>57 min</t>
+          <t>60 min</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>20:29</t>
+          <t>20:34</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>+2.6h</t>
+          <t>+2.7h</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1028,27 +1028,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>21.2h</t>
+          <t>21.3h</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>6.6</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>20:29</t>
+          <t>20:34</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3 min</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>20:32</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1074,27 +1074,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>21.2h</t>
+          <t>21.3h</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>20:32</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>55 min</t>
+          <t>53 min</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>21:27</t>
+          <t>21:32</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>+0.0h</t>
+          <t>+0.2h</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1166,17 +1166,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>21:29</t>
+          <t>21:32</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3 min</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>21:32</t>
+          <t>21:37</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1202,27 +1202,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>22.2h</t>
+          <t>22.3h</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.6</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>21:32</t>
+          <t>21:37</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>57 min</t>
+          <t>60 min</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>22:29</t>
+          <t>22:37</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1247,12 +1247,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>-3.7h</t>
+          <t>-3.6h</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>-2.8h</t>
+          <t>-2.6h</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1284,27 +1284,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2.2h</t>
+          <t>1.9h</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>01:09</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>20 min</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>01:29</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>3 min</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>01:32</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1340,17 +1340,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>01:32</t>
+          <t>01:29</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>21 min</t>
+          <t>19 min</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>01:53</t>
+          <t>01:48</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1375,12 +1375,12 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>-3.9h</t>
+          <t>-4.0h</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>-3.6h</t>
+          <t>-3.7h</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1412,27 +1412,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>3.0h</t>
+          <t>2.9h</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>12.3</t>
+          <t>12.2</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>02:14</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
           <t>02:19</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>3 min</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>02:22</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1458,22 +1458,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3.1h</t>
+          <t>3.0h</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>12.4</t>
+          <t>12.3</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>02:22</t>
+          <t>02:19</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>57 min</t>
+          <t>60 min</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>-3.6h</t>
+          <t>-3.7h</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Flux Standard</t>
+          <t>slew to</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1573,47 +1573,15 @@
           <t>Feige110</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>23:19:58.40</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>-05:09:56.2</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>+4.7h</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>+4.8h</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>11.8</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>1 x 30</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>1 x 30</t>
-        </is>
-      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>Morning standard</t>
-        </is>
-      </c>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1633,44 +1601,80 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10 min</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>03:34</t>
+          <t>03:29</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Arc lamps (HgNeArCdZn)</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
+          <t>Flux Standard</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Feige110</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>23:19:58.40</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>-05:09:56.2</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>+4.8h</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>+4.9h</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>1 x 30</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>1 x 30</t>
+        </is>
+      </c>
       <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Morning standard</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>4.3h</t>
+          <t>4.2h</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>13.6</t>
+          <t>13.5</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>03:34</t>
+          <t>03:29</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1680,12 +1684,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>03:44</t>
+          <t>03:39</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Internal flats</t>
+          <t>Arc lamps (HgNeArCdZn)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -1699,43 +1703,92 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>4.4h</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>13.7</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>03:39</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>10 min</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>03:49</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Internal flats</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>NOTES:</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>- Gap from ~22:29-01:29 HST: no further observable targets in hand</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>- All targets observable at airmass &lt; 2.0 when scheduled</t>
+          <t>- Gap from ~22:37-01:09 HST: no further observable targets in hand</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>- LRIS setup: 560 dichroic, 600/4000 blue grism, 600/7500 red grating (~7200A)</t>
+          <t>- All targets observable at airmass &lt; 2.0 when scheduled</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>- Exposure times from the real LRIS ETC (etc.ucolick.org): S/N=10/pixel per single exposure, 3 exposures min</t>
+          <t>- Keck slews: 5 min base; 20 min when moving from Dec &lt; +20 to Dec &gt; +20</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
+        <is>
+          <t>- LRIS setup: 560 dichroic, 600/4000 blue grism, 600/7500 red grating (~7200A)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>- Exposure times from the real LRIS ETC (etc.ucolick.org): S/N=10/pixel per single exposure, 3 exposures min</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>- MOS (mag&gt;21) targets need ~1-2h once masked (see info column); utilization is target-count-limited: request more targets</t>
         </is>

</xml_diff>